<commit_message>
update structure for multi language
</commit_message>
<xml_diff>
--- a/data/base-text-sop.xlsx
+++ b/data/base-text-sop.xlsx
@@ -8,22 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kauedesousa/Library/Mobile Documents/com~apple~CloudDocs/Work/Rcode/tricot-protocols/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7EDAC46-90A1-2E42-8EB1-0D3EB0818487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEAEC288-D542-464E-82F0-A8C29729AC4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="600" windowWidth="30660" windowHeight="16980" xr2:uid="{CCA2DD50-73A2-AB48-A73E-30174A4C4548}"/>
+    <workbookView xWindow="13420" yWindow="600" windowWidth="17300" windowHeight="16980" xr2:uid="{CCA2DD50-73A2-AB48-A73E-30174A4C4548}"/>
   </bookViews>
   <sheets>
-    <sheet name="text" sheetId="1" r:id="rId1"/>
-    <sheet name="other_resources" sheetId="2" r:id="rId2"/>
+    <sheet name="title" sheetId="3" r:id="rId1"/>
+    <sheet name="text" sheetId="1" r:id="rId2"/>
+    <sheet name="other_resources" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_Toc219906839" localSheetId="0">text!$A$8</definedName>
-    <definedName name="_Toc219906845" localSheetId="0">text!#REF!</definedName>
-    <definedName name="_Toc219906846" localSheetId="0">text!#REF!</definedName>
-    <definedName name="_Toc219906847" localSheetId="0">text!#REF!</definedName>
-    <definedName name="_Toc219906848" localSheetId="0">text!#REF!</definedName>
-    <definedName name="_Toc219906849" localSheetId="0">text!#REF!</definedName>
-    <definedName name="_Toc219906850" localSheetId="0">text!#REF!</definedName>
+    <definedName name="_Toc219906839" localSheetId="1">text!$A$8</definedName>
+    <definedName name="_Toc219906845" localSheetId="1">text!#REF!</definedName>
+    <definedName name="_Toc219906846" localSheetId="1">text!#REF!</definedName>
+    <definedName name="_Toc219906847" localSheetId="1">text!#REF!</definedName>
+    <definedName name="_Toc219906848" localSheetId="1">text!#REF!</definedName>
+    <definedName name="_Toc219906849" localSheetId="1">text!#REF!</definedName>
+    <definedName name="_Toc219906850" localSheetId="1">text!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="113">
   <si>
     <t>en</t>
   </si>
@@ -96,9 +97,6 @@
     <t>Scope</t>
   </si>
   <si>
-    <t>This informed consent form provides a standardised framework to ensure that all participants are adequately informed before taking part in the experiment and associated surveys. It explains the purpose of the data collection, the types of information that will be collected, and how these data may be used, including for research and publication. Participation is entirely voluntary. Participants may decline to answer any question or withdraw from the study at any time, without any negative consequences. Consent is obtained before data collection to ensure transparency, ethical research practice, and respect for participants’ rights. Providing informed consent is a prerequisite for inclusion in all subsequent trial and survey activities. Informed consent template is appended to this SOP.</t>
-  </si>
-  <si>
     <t>scope</t>
   </si>
   <si>
@@ -237,9 +235,6 @@
     <t>trial-observation</t>
   </si>
   <si>
-    <t>Participant registration is conducted during the distribution of trial packages and should be completed for all participants before any subsequent data collection activities can take place. Trial packages should be distributed sufficiently in advance of planting to allow participants adequate time for land preparation and trial establishment. The purpose of registration is to link each participant to a unique trial package and collect the minimum information required for trial management and participant follow-up. Registration activities should remain as brief and efficient as possible, as package distribution is often a busy activity during which project staff must distribute trial materials, explain trial procedures, answer participant questions, and provide implementation guidance. **Completion of participant registration is mandatory for inclusion in subsequent data collection activities and analyses.** During registration, project staff should explain the trial objectives, plot establishment procedures, observation schedule, and participant responsibilities throughout the duration of the trial.</t>
-  </si>
-  <si>
     <t>Participant registration</t>
   </si>
   <si>
@@ -255,9 +250,6 @@
     <t>socioeconomic</t>
   </si>
   <si>
-    <t>Socio-economic data</t>
-  </si>
-  <si>
     <t>socioeconomic-heading</t>
   </si>
   <si>
@@ -286,6 +278,117 @@
   </si>
   <si>
     <t>Other resources and SOPs</t>
+  </si>
+  <si>
+    <t>The informed consent form provides a standardized framework to ensure that all participants are adequately informed before taking part in the experiment and associated surveys. It explains the purpose of the data collection, the types of information that will be collected, and how these data may be used, including for research and publication. Participation is entirely voluntary. Participants may decline to answer any question or withdraw from the study at any time, without any negative consequences. Consent is obtained before data collection to ensure transparency, ethical research practice, and respect for participants’ rights. Providing informed consent is a prerequisite for inclusion in all subsequent trial and survey activities. Informed consent template is appended to this SOP.</t>
+  </si>
+  <si>
+    <t>Socio-economic survey</t>
+  </si>
+  <si>
+    <t>Participant registration is conducted during the distribution of trial packages and should be completed for all participants before any subsequent data collection activities can take place. Trial packages should be distributed sufficiently in advance of planting to allow participants adequate time for land preparation and trial establishment. The purpose of registration is to link each participant to a unique trial package and collect the minimum information required for trial management and participant follow-up. Registration activities should remain as brief and efficient as possible, as package distribution is often a busy activity during which project staff must distribute trial materials, explain trial procedures, answer participant questions, and provide implementation guidance. Completion of participant registration is mandatory for inclusion in subsequent data collection activities and analyses. During registration, project staff should explain the trial objectives, plot establishment procedures, observation schedule, and participant responsibilities throughout the duration of the trial.</t>
+  </si>
+  <si>
+    <t>Escopo</t>
+  </si>
+  <si>
+    <t>Este documento fornece uma visão geral das informações que serão coletadas durante um ensaio em campo com a abordagem tricot. O protocolo apresenta os pontos de coleta de dados durante os ensaios, incluindo as variáveis ​​e características coletadas em cada estágio da cultura. Os agricultores avaliam as variedades em seus ensaios em campo e fornecem observações comparativas, classificando-as com base em seu desempenho relativo ao longo do crescimento e em suas qualidades pós-colheita. Uma visão geral mais detalhada das etapas necessárias para o desenvolvimento de um ensaio participativo em campo usando a abordagem tricot está disponível no seguinte link: https://learn.climmob.net/.</t>
+  </si>
+  <si>
+    <t>**Exclusões:** Este SOP não abrange orientações sobre seleção de genótipos, seleção de participantes, análise estatística avançada, fluxos de trabalho para tomada de decisão em melhoramento genético, procedimentos de análise laboratorial, multiplicação de sementes e protocolos de certificação. Procedimentos específicos relacionados à análise genômica, modelagem climática, regulamentações para envio de sementes ou fenotipagem laboratorial devem ser abordados em SOPs separados, quando aplicável.</t>
+  </si>
+  <si>
+    <t>**Público-alvo:** Este SOP destina-se a melhoristas, agrônomos, funcionários de bancos de germoplasma, ONGs, organizações de agricultores, estudantes e pesquisadores envolvidos na implementação, coordenação e gestão de ensaios de tricotomia e experimentação participativa descentralizada.</t>
+  </si>
+  <si>
+    <t>**Abrangência:** Este SOP descreve os procedimentos e padrões para a implementação de ensaios participativos descentralizados em propriedades rurais utilizando a abordagem tricot. Abrange o planejamento da avaliação, a documentação, o monitoramento e o gerenciamento de dados dos ensaios tricot. O SOP inclui orientações sobre a configuração de questionários digitais, a coleta de dados, os padrões de metadados e os procedimentos básicos de garantia da qualidade para apoiar a geração de dados FAIR. Este SOP visa apoiar a implementação padronizada de ensaios tricot, permitindo, ao mesmo tempo, a adaptação contextual às culturas locais, aos sistemas agrícolas, aos idiomas e aos contextos institucionais.</t>
+  </si>
+  <si>
+    <t>Consentimento</t>
+  </si>
+  <si>
+    <t>O formulário de consentimento livre e esclarecido fornece uma estrutura padronizada para garantir que todos os participantes sejam adequadamente informados antes de participar do experimento e das pesquisas associadas. Ele explica a finalidade da coleta de dados, os tipos de informações que serão coletadas e como esses dados poderão ser usados, inclusive para pesquisa e publicação. A participação é inteiramente voluntária. Os participantes podem se recusar a responder a qualquer pergunta ou desistir do estudo a qualquer momento, sem quaisquer consequências negativas. O consentimento é obtido antes da coleta de dados para garantir transparência, práticas de pesquisa éticas e respeito aos direitos dos participantes. O fornecimento do consentimento livre e esclarecido é um pré-requisito para a inclusão em todas as atividades subsequentes do ensaio clínico e das pesquisas. O modelo de consentimento livre e esclarecido está anexado a este SOP.</t>
+  </si>
+  <si>
+    <t>Desenho experimental</t>
+  </si>
+  <si>
+    <t>Todas as parcelas são identificadas pelas letras A, B e C. As parcelas devem ser estabelecidas na mesma data de plantio e seguir as mesmas dimensões e práticas de manejo. O tamanho das parcelas deve seguir as recomendações da equipe de implementação local e ser adequado à cultura e ao sistema de cultivo. As informações sobre as dimensões das parcelas devem ser registradas nos metadados do ensaio. As três parcelas devem ser localizadas no mesmo campo, sempre que possível, para garantir a exposição a condições ambientais e de manejo semelhantes. Se houver área suficiente disponível, os agricultores são incentivados a estabelecer uma parcela adicional de sua variedade local preferida ou comumente cultivada ("Local"), utilizando a mesma data de plantio, tamanho e práticas de manejo. Embora a parcela Local não faça parte do delineamento principal do experimento, ela pode ser incluída na avaliação de final de safra, na qual os participantes são questionados sobre se a variedade local apresentou desempenho melhor ou pior do que as opções A, B e C.</t>
+  </si>
+  <si>
+    <t>Standard operating procedures for data collection and implementation of on-farm trials with the tricot approach</t>
+  </si>
+  <si>
+    <t>Procedimentos operacionais padrão para coleta de dados e implementação de ensaios experimentais em fazendas com a abordagem tricot</t>
+  </si>
+  <si>
+    <t>Versão</t>
+  </si>
+  <si>
+    <t>Version</t>
+  </si>
+  <si>
+    <t>Crop</t>
+  </si>
+  <si>
+    <t>Taxa</t>
+  </si>
+  <si>
+    <t>Authors</t>
+  </si>
+  <si>
+    <t>Institutions</t>
+  </si>
+  <si>
+    <t>Traits</t>
+  </si>
+  <si>
+    <t>Data collection moments</t>
+  </si>
+  <si>
+    <t>Cultivo</t>
+  </si>
+  <si>
+    <t>Taxonomia</t>
+  </si>
+  <si>
+    <t>Autores</t>
+  </si>
+  <si>
+    <t>Instituições</t>
+  </si>
+  <si>
+    <t>Atributos</t>
+  </si>
+  <si>
+    <t>Estádios de coleta de dados</t>
+  </si>
+  <si>
+    <t>Question name</t>
+  </si>
+  <si>
+    <t>Question description</t>
+  </si>
+  <si>
+    <t>Nome da pergunta</t>
+  </si>
+  <si>
+    <t>Descrição</t>
+  </si>
+  <si>
+    <t>Resource</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>Recurso</t>
+  </si>
+  <si>
+    <t>This document is also available in</t>
+  </si>
+  <si>
+    <t>Este documento também está disponível em</t>
   </si>
 </sst>
 </file>
@@ -342,7 +445,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
@@ -351,6 +454,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -686,244 +792,133 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB5FF5ED-AA91-F847-8546-368AFFC4F6A2}">
-  <dimension ref="A1:F27"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70DB7E77-C0DE-BB4E-8530-DD7ED990578A}">
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="31.33203125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="91" style="3" customWidth="1"/>
-    <col min="3" max="16384" width="10.83203125" style="3"/>
+    <col min="1" max="1" width="23.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:5" ht="102" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="119" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="119" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="85" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="51" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="138" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="170" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="51" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="68" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="51" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="51" x14ac:dyDescent="0.2">
-      <c r="A16" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="34" x14ac:dyDescent="0.2">
-      <c r="A17" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="17" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="180" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="204" x14ac:dyDescent="0.2">
-      <c r="A21" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="238" x14ac:dyDescent="0.2">
-      <c r="A23" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A24" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="187" x14ac:dyDescent="0.2">
-      <c r="A25" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A26" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A27" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>77</v>
+        <v>88</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>93</v>
+      </c>
+      <c r="B5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B6" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B8" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>97</v>
+      </c>
+      <c r="B9" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>111</v>
+      </c>
+      <c r="B10" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>104</v>
+      </c>
+      <c r="B11" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>105</v>
+      </c>
+      <c r="B12" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>108</v>
+      </c>
+      <c r="B13" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>109</v>
+      </c>
+      <c r="B14" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -932,6 +927,280 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB5FF5ED-AA91-F847-8546-368AFFC4F6A2}">
+  <dimension ref="A1:F27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="31.33203125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="49.83203125" style="3" customWidth="1"/>
+    <col min="3" max="3" width="43.6640625" style="4" customWidth="1"/>
+    <col min="4" max="16384" width="10.83203125" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="251" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="306" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="221" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="136" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="404" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="102" x14ac:dyDescent="0.2">
+      <c r="A13" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="119" x14ac:dyDescent="0.2">
+      <c r="A14" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="85" x14ac:dyDescent="0.2">
+      <c r="A15" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="85" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="51" x14ac:dyDescent="0.2">
+      <c r="A17" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="17" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="180" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="372" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="409.6" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="340" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4041A62-4750-304C-A0F2-6428C3DB8928}">
   <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -943,7 +1212,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -963,98 +1232,98 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>